<commit_message>
Add Svs profils (#170)
* rm index file and add svs profiles

* ajout description 6e8ff2fd614f58e1c137933fee8931f128b5f797
</commit_message>
<xml_diff>
--- a/ig/main/StructureDefinition-as-dp-practitioner.xlsx
+++ b/ig/main/StructureDefinition-as-dp-practitioner.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-02-07T08:22:38+00:00</t>
+    <t>2024-02-08T15:43:07+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -745,7 +745,8 @@
 </t>
   </si>
   <si>
-    <t>Description of identifier</t>
+    <t>Type d’identifiant national de la personne physique (typeIdNat_PP),
+Les codes ADELI, RPPS et IDNPS proviennent du system  http://interopsante.org/fhir/CodeSystem/fr-v2-0203 ; Les codes 1, 3, 4, 5, 6 proviennent du system : https://mos.esante.gouv.fr/NOS/TRE_G08-TypeIdentifiantPersonne/FHIR/TRE-G08-TypeIdentifiantPersonne</t>
   </si>
   <si>
     <t>A coded type for the identifier that can be used to determine which identifier to use for a specific purpose.</t>
@@ -1015,8 +1016,7 @@
     <t>Practitioner.identifier:idNatPs.type</t>
   </si>
   <si>
-    <t>Type d’identifiant national de la personne physique (typeIdNat_PP),
-Les codes ADELI, RPPS et IDNPS proviennent du system  http://interopsante.org/fhir/CodeSystem/fr-v2-0203 ; Les codes 1, 3, 4, 5, 6 proviennent du system : https://mos.esante.gouv.fr/NOS/TRE_G08-TypeIdentifiantPersonne/FHIR/TRE-G08-TypeIdentifiantPersonne</t>
+    <t>Description of identifier</t>
   </si>
   <si>
     <t>&lt;valueCodeableConcept xmlns="http://hl7.org/fhir"&gt;
@@ -10980,7 +10980,7 @@
         <v>231</v>
       </c>
       <c r="L68" t="s" s="2">
-        <v>232</v>
+        <v>319</v>
       </c>
       <c r="M68" t="s" s="2">
         <v>233</v>
@@ -13034,7 +13034,7 @@
         <v>231</v>
       </c>
       <c r="L88" t="s" s="2">
-        <v>232</v>
+        <v>319</v>
       </c>
       <c r="M88" t="s" s="2">
         <v>233</v>
@@ -15088,7 +15088,7 @@
         <v>231</v>
       </c>
       <c r="L108" t="s" s="2">
-        <v>232</v>
+        <v>319</v>
       </c>
       <c r="M108" t="s" s="2">
         <v>233</v>

</xml_diff>

<commit_message>
Amélioration display ressource (#174)
* update

* rm degreeR[x] slices

* add downloads page

* update exercicePro short

* change slice name in DpPractitioner 59b4c74c708effed9f63d8c54a5509d7bb32457f
</commit_message>
<xml_diff>
--- a/ig/main/StructureDefinition-as-dp-practitioner.xlsx
+++ b/ig/main/StructureDefinition-as-dp-practitioner.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21335" uniqueCount="1205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21335" uniqueCount="1206">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-02-16T10:57:00+00:00</t>
+    <t>2024-02-16T18:38:53+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -2888,426 +2888,424 @@
     <t>[Donnée restreinte] : Lieu de formation pour l'obtention du diplôme (lieuFormation).</t>
   </si>
   <si>
-    <t>Practitioner.qualification:profession</t>
+    <t>Practitioner.qualification:exercicePro</t>
+  </si>
+  <si>
+    <t>exercicePro</t>
+  </si>
+  <si>
+    <t>exercicePro : exercice professionnel décrivant la profession exercée, l'identité d'exercice d'un professionnel et le cadre de son exercice (civil, militaire, etc.).</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.id</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.extension</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.modifierExtension</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.identifier</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.id</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.extension</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR36</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR36.id</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR36.extension</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR36.system</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR36.version</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR36.code</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR36.display</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR36.userSelected</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR47</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR47.id</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR47.extension</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR47.system</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR47.version</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR47.code</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR47.display</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR47.userSelected</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR48</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR48.id</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR48.extension</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR48.system</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR48.version</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR48.code</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR48.display</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR48.userSelected</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR49</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR49.id</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR49.extension</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR49.system</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR49.version</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR49.code</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR49.display</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR49.userSelected</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR50</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR50.id</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR50.extension</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR50.system</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR50.version</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR50.code</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR50.display</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR50.userSelected</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR51</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR51.id</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR51.extension</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR51.system</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR51.version</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR51.code</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR51.display</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR51.userSelected</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR52</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR52.id</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR52.extension</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR52.system</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR52.version</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR52.code</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR52.display</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR52.userSelected</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR53</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR53.id</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR53.extension</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR53.system</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR53.version</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR53.code</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR53.display</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR53.userSelected</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR54</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR54.id</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR54.extension</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR54.system</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR54.version</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR54.code</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR54.display</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR54.userSelected</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR55</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR55.id</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR55.extension</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR55.system</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR55.version</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR55.code</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR55.display</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR55.userSelected</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR56</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR56.id</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR56.extension</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR56.system</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR56.version</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR56.code</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR56.display</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR56.userSelected</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR57</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR57.id</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR57.extension</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR57.system</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR57.version</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR57.code</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR57.display</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR57.userSelected</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR58</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR58.id</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR58.extension</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR58.system</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR58.version</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR58.code</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR58.display</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR58.userSelected</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR226</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR226.id</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR226.extension</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR226.system</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR226.version</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR226.code</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR226.display</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:degreeR226.userSelected</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:categorieProfession</t>
+  </si>
+  <si>
+    <t>categorieProfession</t>
+  </si>
+  <si>
+    <t>Catégorie professionnelle indiquant si le professionnel exerce sa profession en tant que Militaire, Civil, Fonctionnaire ou Etudiant (categorieProfessionnelle).</t>
+  </si>
+  <si>
+    <t>https://mos.esante.gouv.fr/NOS/JDV_J89-CategorieProfessionnelle-RASS/FHIR/JDV-J89-CategorieProfessionnelle-RASS</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.code.coding:profession</t>
   </si>
   <si>
     <t>profession</t>
   </si>
   <si>
-    <t>profession : Profession exercée ou future profession de l'étudiant.
-categorieProfessionnelle : Indique si le professionnel exerce sa profession en tant que :
-M: Militaire
-C: Civil
-F: Fonctionnaire
-E: Etudiant</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.id</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.extension</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.modifierExtension</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.identifier</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.id</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.extension</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR36</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR36.id</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR36.extension</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR36.system</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR36.version</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR36.code</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR36.display</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR36.userSelected</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR47</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR47.id</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR47.extension</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR47.system</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR47.version</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR47.code</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR47.display</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR47.userSelected</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR48</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR48.id</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR48.extension</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR48.system</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR48.version</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR48.code</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR48.display</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR48.userSelected</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR49</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR49.id</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR49.extension</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR49.system</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR49.version</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR49.code</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR49.display</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR49.userSelected</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR50</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR50.id</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR50.extension</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR50.system</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR50.version</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR50.code</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR50.display</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR50.userSelected</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR51</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR51.id</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR51.extension</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR51.system</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR51.version</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR51.code</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR51.display</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR51.userSelected</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR52</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR52.id</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR52.extension</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR52.system</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR52.version</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR52.code</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR52.display</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR52.userSelected</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR53</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR53.id</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR53.extension</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR53.system</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR53.version</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR53.code</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR53.display</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR53.userSelected</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR54</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR54.id</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR54.extension</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR54.system</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR54.version</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR54.code</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR54.display</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR54.userSelected</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR55</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR55.id</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR55.extension</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR55.system</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR55.version</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR55.code</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR55.display</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR55.userSelected</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR56</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR56.id</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR56.extension</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR56.system</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR56.version</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR56.code</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR56.display</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR56.userSelected</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR57</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR57.id</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR57.extension</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR57.system</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR57.version</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR57.code</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR57.display</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR57.userSelected</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR58</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR58.id</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR58.extension</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR58.system</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR58.version</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR58.code</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR58.display</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR58.userSelected</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR226</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR226.id</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR226.extension</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR226.system</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR226.version</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR226.code</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR226.display</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:degreeR226.userSelected</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:categorieProfession</t>
-  </si>
-  <si>
-    <t>categorieProfession</t>
-  </si>
-  <si>
-    <t>Catégorie professionnelle indiqant si le professionnel exerce sa profession en tant que Militaire, Civil, Fonctionnaire ou Etudiant (categorieProfessionnelle).</t>
-  </si>
-  <si>
-    <t>https://mos.esante.gouv.fr/NOS/JDV_J89-CategorieProfessionnelle-RASS/FHIR/JDV-J89-CategorieProfessionnelle-RASS</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.code.coding:profession</t>
-  </si>
-  <si>
     <t>Profession exercée : de santé (professionSante) TRE G15, du social (professionSocial) TRE R94, à usage de titre professionnel (usagerTitre) TRE R95, ou autre profession (autreProfession) TRE R291</t>
   </si>
   <si>
     <t>https://mos.esante.gouv.fr/NOS/JDV_J106-EnsembleProfession-RASS/FHIR/JDV-J106-EnsembleProfession-RASS</t>
   </si>
   <si>
-    <t>Practitioner.qualification:profession.code.text</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.period</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.period.id</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.period.extension</t>
-  </si>
-  <si>
-    <t>Practitioner.qualification:profession.period.start</t>
+    <t>Practitioner.qualification:exercicePro.code.text</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.period</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.period.id</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.period.extension</t>
+  </si>
+  <si>
+    <t>Practitioner.qualification:exercicePro.period.start</t>
   </si>
   <si>
     <t>[Donnée restreinte] : Date à partir de laquelle le professionnel n’exerce plus cette profession (dateFinEffetExercice).</t>
   </si>
   <si>
-    <t>Practitioner.qualification:profession.period.end</t>
+    <t>Practitioner.qualification:exercicePro.period.end</t>
   </si>
   <si>
     <t>End time with inclusive boundary, if not ongoing</t>
   </si>
   <si>
-    <t>Practitioner.qualification:profession.issuer</t>
+    <t>Practitioner.qualification:exercicePro.issuer</t>
   </si>
   <si>
     <t>Practitioner.qualification:savoirFaire</t>
@@ -46129,7 +46127,7 @@
         <v>74</v>
       </c>
       <c r="G410" t="s" s="2">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H410" t="s" s="2">
         <v>73</v>
@@ -46953,7 +46951,7 @@
         <v>74</v>
       </c>
       <c r="G418" t="s" s="2">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H418" t="s" s="2">
         <v>73</v>
@@ -47777,7 +47775,7 @@
         <v>74</v>
       </c>
       <c r="G426" t="s" s="2">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H426" t="s" s="2">
         <v>73</v>
@@ -48601,7 +48599,7 @@
         <v>74</v>
       </c>
       <c r="G434" t="s" s="2">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H434" t="s" s="2">
         <v>73</v>
@@ -49425,7 +49423,7 @@
         <v>74</v>
       </c>
       <c r="G442" t="s" s="2">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H442" t="s" s="2">
         <v>73</v>
@@ -50249,7 +50247,7 @@
         <v>74</v>
       </c>
       <c r="G450" t="s" s="2">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H450" t="s" s="2">
         <v>73</v>
@@ -51073,7 +51071,7 @@
         <v>74</v>
       </c>
       <c r="G458" t="s" s="2">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H458" t="s" s="2">
         <v>73</v>
@@ -51897,7 +51895,7 @@
         <v>74</v>
       </c>
       <c r="G466" t="s" s="2">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H466" t="s" s="2">
         <v>73</v>
@@ -52721,7 +52719,7 @@
         <v>74</v>
       </c>
       <c r="G474" t="s" s="2">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H474" t="s" s="2">
         <v>73</v>
@@ -53545,7 +53543,7 @@
         <v>74</v>
       </c>
       <c r="G482" t="s" s="2">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H482" t="s" s="2">
         <v>73</v>
@@ -54369,7 +54367,7 @@
         <v>74</v>
       </c>
       <c r="G490" t="s" s="2">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H490" t="s" s="2">
         <v>73</v>
@@ -55193,7 +55191,7 @@
         <v>74</v>
       </c>
       <c r="G498" t="s" s="2">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H498" t="s" s="2">
         <v>73</v>
@@ -56017,7 +56015,7 @@
         <v>74</v>
       </c>
       <c r="G506" t="s" s="2">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H506" t="s" s="2">
         <v>73</v>
@@ -56841,7 +56839,7 @@
         <v>74</v>
       </c>
       <c r="G514" t="s" s="2">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H514" t="s" s="2">
         <v>73</v>
@@ -57759,7 +57757,7 @@
         <v>597</v>
       </c>
       <c r="C523" t="s" s="2">
-        <v>928</v>
+        <v>1055</v>
       </c>
       <c r="D523" t="s" s="2">
         <v>73</v>
@@ -57784,7 +57782,7 @@
         <v>140</v>
       </c>
       <c r="L523" t="s" s="2">
-        <v>1055</v>
+        <v>1056</v>
       </c>
       <c r="M523" t="s" s="2">
         <v>243</v>
@@ -57822,7 +57820,7 @@
       </c>
       <c r="Y523" s="2"/>
       <c r="Z523" t="s" s="2">
-        <v>1056</v>
+        <v>1057</v>
       </c>
       <c r="AA523" t="s" s="2">
         <v>73</v>
@@ -57857,7 +57855,7 @@
     </row>
     <row r="524" hidden="true">
       <c r="A524" t="s" s="2">
-        <v>1057</v>
+        <v>1058</v>
       </c>
       <c r="B524" t="s" s="2">
         <v>761</v>
@@ -57961,7 +57959,7 @@
     </row>
     <row r="525" hidden="true">
       <c r="A525" t="s" s="2">
-        <v>1058</v>
+        <v>1059</v>
       </c>
       <c r="B525" t="s" s="2">
         <v>762</v>
@@ -58065,7 +58063,7 @@
     </row>
     <row r="526" hidden="true">
       <c r="A526" t="s" s="2">
-        <v>1059</v>
+        <v>1060</v>
       </c>
       <c r="B526" t="s" s="2">
         <v>906</v>
@@ -58165,7 +58163,7 @@
     </row>
     <row r="527" hidden="true">
       <c r="A527" t="s" s="2">
-        <v>1060</v>
+        <v>1061</v>
       </c>
       <c r="B527" t="s" s="2">
         <v>908</v>
@@ -58267,7 +58265,7 @@
     </row>
     <row r="528" hidden="true">
       <c r="A528" t="s" s="2">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="B528" t="s" s="2">
         <v>910</v>
@@ -58296,7 +58294,7 @@
         <v>911</v>
       </c>
       <c r="L528" t="s" s="2">
-        <v>1062</v>
+        <v>1063</v>
       </c>
       <c r="M528" t="s" s="2">
         <v>913</v>
@@ -58369,7 +58367,7 @@
     </row>
     <row r="529" hidden="true">
       <c r="A529" t="s" s="2">
-        <v>1063</v>
+        <v>1064</v>
       </c>
       <c r="B529" t="s" s="2">
         <v>918</v>
@@ -58398,7 +58396,7 @@
         <v>911</v>
       </c>
       <c r="L529" t="s" s="2">
-        <v>1064</v>
+        <v>1065</v>
       </c>
       <c r="M529" t="s" s="2">
         <v>920</v>
@@ -58473,7 +58471,7 @@
     </row>
     <row r="530" hidden="true">
       <c r="A530" t="s" s="2">
-        <v>1065</v>
+        <v>1066</v>
       </c>
       <c r="B530" t="s" s="2">
         <v>766</v>
@@ -58575,13 +58573,13 @@
     </row>
     <row r="531" hidden="true">
       <c r="A531" t="s" s="2">
-        <v>1066</v>
+        <v>1067</v>
       </c>
       <c r="B531" t="s" s="2">
         <v>573</v>
       </c>
       <c r="C531" t="s" s="2">
-        <v>1067</v>
+        <v>1068</v>
       </c>
       <c r="D531" t="s" s="2">
         <v>73</v>
@@ -58606,7 +58604,7 @@
         <v>574</v>
       </c>
       <c r="L531" t="s" s="2">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="M531" t="s" s="2">
         <v>576</v>
@@ -58677,7 +58675,7 @@
     </row>
     <row r="532" hidden="true">
       <c r="A532" t="s" s="2">
-        <v>1069</v>
+        <v>1070</v>
       </c>
       <c r="B532" t="s" s="2">
         <v>578</v>
@@ -58777,7 +58775,7 @@
     </row>
     <row r="533" hidden="true">
       <c r="A533" t="s" s="2">
-        <v>1070</v>
+        <v>1071</v>
       </c>
       <c r="B533" t="s" s="2">
         <v>579</v>
@@ -58879,7 +58877,7 @@
     </row>
     <row r="534" hidden="true">
       <c r="A534" t="s" s="2">
-        <v>1071</v>
+        <v>1072</v>
       </c>
       <c r="B534" t="s" s="2">
         <v>580</v>
@@ -58983,7 +58981,7 @@
     </row>
     <row r="535" hidden="true">
       <c r="A535" t="s" s="2">
-        <v>1072</v>
+        <v>1073</v>
       </c>
       <c r="B535" t="s" s="2">
         <v>585</v>
@@ -59085,7 +59083,7 @@
     </row>
     <row r="536" hidden="true">
       <c r="A536" t="s" s="2">
-        <v>1073</v>
+        <v>1074</v>
       </c>
       <c r="B536" t="s" s="2">
         <v>589</v>
@@ -59187,7 +59185,7 @@
     </row>
     <row r="537" hidden="true">
       <c r="A537" t="s" s="2">
-        <v>1074</v>
+        <v>1075</v>
       </c>
       <c r="B537" t="s" s="2">
         <v>595</v>
@@ -59287,7 +59285,7 @@
     </row>
     <row r="538" hidden="true">
       <c r="A538" t="s" s="2">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="B538" t="s" s="2">
         <v>596</v>
@@ -59389,7 +59387,7 @@
     </row>
     <row r="539" hidden="true">
       <c r="A539" t="s" s="2">
-        <v>1076</v>
+        <v>1077</v>
       </c>
       <c r="B539" t="s" s="2">
         <v>597</v>
@@ -59491,7 +59489,7 @@
     </row>
     <row r="540" hidden="true">
       <c r="A540" t="s" s="2">
-        <v>1077</v>
+        <v>1078</v>
       </c>
       <c r="B540" t="s" s="2">
         <v>597</v>
@@ -59507,7 +59505,7 @@
         <v>74</v>
       </c>
       <c r="G540" t="s" s="2">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H540" t="s" s="2">
         <v>73</v>
@@ -59595,7 +59593,7 @@
     </row>
     <row r="541" hidden="true">
       <c r="A541" t="s" s="2">
-        <v>1078</v>
+        <v>1079</v>
       </c>
       <c r="B541" t="s" s="2">
         <v>603</v>
@@ -59695,7 +59693,7 @@
     </row>
     <row r="542" hidden="true">
       <c r="A542" t="s" s="2">
-        <v>1079</v>
+        <v>1080</v>
       </c>
       <c r="B542" t="s" s="2">
         <v>605</v>
@@ -59797,7 +59795,7 @@
     </row>
     <row r="543" hidden="true">
       <c r="A543" t="s" s="2">
-        <v>1080</v>
+        <v>1081</v>
       </c>
       <c r="B543" t="s" s="2">
         <v>607</v>
@@ -59901,7 +59899,7 @@
     </row>
     <row r="544" hidden="true">
       <c r="A544" t="s" s="2">
-        <v>1081</v>
+        <v>1082</v>
       </c>
       <c r="B544" t="s" s="2">
         <v>611</v>
@@ -60003,7 +60001,7 @@
     </row>
     <row r="545" hidden="true">
       <c r="A545" t="s" s="2">
-        <v>1082</v>
+        <v>1083</v>
       </c>
       <c r="B545" t="s" s="2">
         <v>613</v>
@@ -60107,7 +60105,7 @@
     </row>
     <row r="546" hidden="true">
       <c r="A546" t="s" s="2">
-        <v>1083</v>
+        <v>1084</v>
       </c>
       <c r="B546" t="s" s="2">
         <v>615</v>
@@ -60211,7 +60209,7 @@
     </row>
     <row r="547" hidden="true">
       <c r="A547" t="s" s="2">
-        <v>1084</v>
+        <v>1085</v>
       </c>
       <c r="B547" t="s" s="2">
         <v>617</v>
@@ -60315,7 +60313,7 @@
     </row>
     <row r="548" hidden="true">
       <c r="A548" t="s" s="2">
-        <v>1085</v>
+        <v>1086</v>
       </c>
       <c r="B548" t="s" s="2">
         <v>597</v>
@@ -60331,7 +60329,7 @@
         <v>74</v>
       </c>
       <c r="G548" t="s" s="2">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H548" t="s" s="2">
         <v>73</v>
@@ -60419,7 +60417,7 @@
     </row>
     <row r="549" hidden="true">
       <c r="A549" t="s" s="2">
-        <v>1086</v>
+        <v>1087</v>
       </c>
       <c r="B549" t="s" s="2">
         <v>603</v>
@@ -60519,7 +60517,7 @@
     </row>
     <row r="550" hidden="true">
       <c r="A550" t="s" s="2">
-        <v>1087</v>
+        <v>1088</v>
       </c>
       <c r="B550" t="s" s="2">
         <v>605</v>
@@ -60621,7 +60619,7 @@
     </row>
     <row r="551" hidden="true">
       <c r="A551" t="s" s="2">
-        <v>1088</v>
+        <v>1089</v>
       </c>
       <c r="B551" t="s" s="2">
         <v>607</v>
@@ -60725,7 +60723,7 @@
     </row>
     <row r="552" hidden="true">
       <c r="A552" t="s" s="2">
-        <v>1089</v>
+        <v>1090</v>
       </c>
       <c r="B552" t="s" s="2">
         <v>611</v>
@@ -60827,7 +60825,7 @@
     </row>
     <row r="553" hidden="true">
       <c r="A553" t="s" s="2">
-        <v>1090</v>
+        <v>1091</v>
       </c>
       <c r="B553" t="s" s="2">
         <v>613</v>
@@ -60931,7 +60929,7 @@
     </row>
     <row r="554" hidden="true">
       <c r="A554" t="s" s="2">
-        <v>1091</v>
+        <v>1092</v>
       </c>
       <c r="B554" t="s" s="2">
         <v>615</v>
@@ -61035,7 +61033,7 @@
     </row>
     <row r="555" hidden="true">
       <c r="A555" t="s" s="2">
-        <v>1092</v>
+        <v>1093</v>
       </c>
       <c r="B555" t="s" s="2">
         <v>617</v>
@@ -61139,7 +61137,7 @@
     </row>
     <row r="556" hidden="true">
       <c r="A556" t="s" s="2">
-        <v>1093</v>
+        <v>1094</v>
       </c>
       <c r="B556" t="s" s="2">
         <v>597</v>
@@ -61155,7 +61153,7 @@
         <v>74</v>
       </c>
       <c r="G556" t="s" s="2">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H556" t="s" s="2">
         <v>73</v>
@@ -61243,7 +61241,7 @@
     </row>
     <row r="557" hidden="true">
       <c r="A557" t="s" s="2">
-        <v>1094</v>
+        <v>1095</v>
       </c>
       <c r="B557" t="s" s="2">
         <v>603</v>
@@ -61343,7 +61341,7 @@
     </row>
     <row r="558" hidden="true">
       <c r="A558" t="s" s="2">
-        <v>1095</v>
+        <v>1096</v>
       </c>
       <c r="B558" t="s" s="2">
         <v>605</v>
@@ -61445,7 +61443,7 @@
     </row>
     <row r="559" hidden="true">
       <c r="A559" t="s" s="2">
-        <v>1096</v>
+        <v>1097</v>
       </c>
       <c r="B559" t="s" s="2">
         <v>607</v>
@@ -61549,7 +61547,7 @@
     </row>
     <row r="560" hidden="true">
       <c r="A560" t="s" s="2">
-        <v>1097</v>
+        <v>1098</v>
       </c>
       <c r="B560" t="s" s="2">
         <v>611</v>
@@ -61651,7 +61649,7 @@
     </row>
     <row r="561" hidden="true">
       <c r="A561" t="s" s="2">
-        <v>1098</v>
+        <v>1099</v>
       </c>
       <c r="B561" t="s" s="2">
         <v>613</v>
@@ -61755,7 +61753,7 @@
     </row>
     <row r="562" hidden="true">
       <c r="A562" t="s" s="2">
-        <v>1099</v>
+        <v>1100</v>
       </c>
       <c r="B562" t="s" s="2">
         <v>615</v>
@@ -61859,7 +61857,7 @@
     </row>
     <row r="563" hidden="true">
       <c r="A563" t="s" s="2">
-        <v>1100</v>
+        <v>1101</v>
       </c>
       <c r="B563" t="s" s="2">
         <v>617</v>
@@ -61963,7 +61961,7 @@
     </row>
     <row r="564" hidden="true">
       <c r="A564" t="s" s="2">
-        <v>1101</v>
+        <v>1102</v>
       </c>
       <c r="B564" t="s" s="2">
         <v>597</v>
@@ -61979,7 +61977,7 @@
         <v>74</v>
       </c>
       <c r="G564" t="s" s="2">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H564" t="s" s="2">
         <v>73</v>
@@ -62067,7 +62065,7 @@
     </row>
     <row r="565" hidden="true">
       <c r="A565" t="s" s="2">
-        <v>1102</v>
+        <v>1103</v>
       </c>
       <c r="B565" t="s" s="2">
         <v>603</v>
@@ -62167,7 +62165,7 @@
     </row>
     <row r="566" hidden="true">
       <c r="A566" t="s" s="2">
-        <v>1103</v>
+        <v>1104</v>
       </c>
       <c r="B566" t="s" s="2">
         <v>605</v>
@@ -62269,7 +62267,7 @@
     </row>
     <row r="567" hidden="true">
       <c r="A567" t="s" s="2">
-        <v>1104</v>
+        <v>1105</v>
       </c>
       <c r="B567" t="s" s="2">
         <v>607</v>
@@ -62373,7 +62371,7 @@
     </row>
     <row r="568" hidden="true">
       <c r="A568" t="s" s="2">
-        <v>1105</v>
+        <v>1106</v>
       </c>
       <c r="B568" t="s" s="2">
         <v>611</v>
@@ -62475,7 +62473,7 @@
     </row>
     <row r="569" hidden="true">
       <c r="A569" t="s" s="2">
-        <v>1106</v>
+        <v>1107</v>
       </c>
       <c r="B569" t="s" s="2">
         <v>613</v>
@@ -62579,7 +62577,7 @@
     </row>
     <row r="570" hidden="true">
       <c r="A570" t="s" s="2">
-        <v>1107</v>
+        <v>1108</v>
       </c>
       <c r="B570" t="s" s="2">
         <v>615</v>
@@ -62683,7 +62681,7 @@
     </row>
     <row r="571" hidden="true">
       <c r="A571" t="s" s="2">
-        <v>1108</v>
+        <v>1109</v>
       </c>
       <c r="B571" t="s" s="2">
         <v>617</v>
@@ -62787,7 +62785,7 @@
     </row>
     <row r="572" hidden="true">
       <c r="A572" t="s" s="2">
-        <v>1109</v>
+        <v>1110</v>
       </c>
       <c r="B572" t="s" s="2">
         <v>597</v>
@@ -62803,7 +62801,7 @@
         <v>74</v>
       </c>
       <c r="G572" t="s" s="2">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H572" t="s" s="2">
         <v>73</v>
@@ -62891,7 +62889,7 @@
     </row>
     <row r="573" hidden="true">
       <c r="A573" t="s" s="2">
-        <v>1110</v>
+        <v>1111</v>
       </c>
       <c r="B573" t="s" s="2">
         <v>603</v>
@@ -62991,7 +62989,7 @@
     </row>
     <row r="574" hidden="true">
       <c r="A574" t="s" s="2">
-        <v>1111</v>
+        <v>1112</v>
       </c>
       <c r="B574" t="s" s="2">
         <v>605</v>
@@ -63093,7 +63091,7 @@
     </row>
     <row r="575" hidden="true">
       <c r="A575" t="s" s="2">
-        <v>1112</v>
+        <v>1113</v>
       </c>
       <c r="B575" t="s" s="2">
         <v>607</v>
@@ -63197,7 +63195,7 @@
     </row>
     <row r="576" hidden="true">
       <c r="A576" t="s" s="2">
-        <v>1113</v>
+        <v>1114</v>
       </c>
       <c r="B576" t="s" s="2">
         <v>611</v>
@@ -63299,7 +63297,7 @@
     </row>
     <row r="577" hidden="true">
       <c r="A577" t="s" s="2">
-        <v>1114</v>
+        <v>1115</v>
       </c>
       <c r="B577" t="s" s="2">
         <v>613</v>
@@ -63403,7 +63401,7 @@
     </row>
     <row r="578" hidden="true">
       <c r="A578" t="s" s="2">
-        <v>1115</v>
+        <v>1116</v>
       </c>
       <c r="B578" t="s" s="2">
         <v>615</v>
@@ -63507,7 +63505,7 @@
     </row>
     <row r="579" hidden="true">
       <c r="A579" t="s" s="2">
-        <v>1116</v>
+        <v>1117</v>
       </c>
       <c r="B579" t="s" s="2">
         <v>617</v>
@@ -63611,7 +63609,7 @@
     </row>
     <row r="580" hidden="true">
       <c r="A580" t="s" s="2">
-        <v>1117</v>
+        <v>1118</v>
       </c>
       <c r="B580" t="s" s="2">
         <v>597</v>
@@ -63627,7 +63625,7 @@
         <v>74</v>
       </c>
       <c r="G580" t="s" s="2">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H580" t="s" s="2">
         <v>73</v>
@@ -63715,7 +63713,7 @@
     </row>
     <row r="581" hidden="true">
       <c r="A581" t="s" s="2">
-        <v>1118</v>
+        <v>1119</v>
       </c>
       <c r="B581" t="s" s="2">
         <v>603</v>
@@ -63815,7 +63813,7 @@
     </row>
     <row r="582" hidden="true">
       <c r="A582" t="s" s="2">
-        <v>1119</v>
+        <v>1120</v>
       </c>
       <c r="B582" t="s" s="2">
         <v>605</v>
@@ -63917,7 +63915,7 @@
     </row>
     <row r="583" hidden="true">
       <c r="A583" t="s" s="2">
-        <v>1120</v>
+        <v>1121</v>
       </c>
       <c r="B583" t="s" s="2">
         <v>607</v>
@@ -64021,7 +64019,7 @@
     </row>
     <row r="584" hidden="true">
       <c r="A584" t="s" s="2">
-        <v>1121</v>
+        <v>1122</v>
       </c>
       <c r="B584" t="s" s="2">
         <v>611</v>
@@ -64123,7 +64121,7 @@
     </row>
     <row r="585" hidden="true">
       <c r="A585" t="s" s="2">
-        <v>1122</v>
+        <v>1123</v>
       </c>
       <c r="B585" t="s" s="2">
         <v>613</v>
@@ -64227,7 +64225,7 @@
     </row>
     <row r="586" hidden="true">
       <c r="A586" t="s" s="2">
-        <v>1123</v>
+        <v>1124</v>
       </c>
       <c r="B586" t="s" s="2">
         <v>615</v>
@@ -64331,7 +64329,7 @@
     </row>
     <row r="587" hidden="true">
       <c r="A587" t="s" s="2">
-        <v>1124</v>
+        <v>1125</v>
       </c>
       <c r="B587" t="s" s="2">
         <v>617</v>
@@ -64435,7 +64433,7 @@
     </row>
     <row r="588" hidden="true">
       <c r="A588" t="s" s="2">
-        <v>1125</v>
+        <v>1126</v>
       </c>
       <c r="B588" t="s" s="2">
         <v>597</v>
@@ -64451,7 +64449,7 @@
         <v>74</v>
       </c>
       <c r="G588" t="s" s="2">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H588" t="s" s="2">
         <v>73</v>
@@ -64539,7 +64537,7 @@
     </row>
     <row r="589" hidden="true">
       <c r="A589" t="s" s="2">
-        <v>1126</v>
+        <v>1127</v>
       </c>
       <c r="B589" t="s" s="2">
         <v>603</v>
@@ -64639,7 +64637,7 @@
     </row>
     <row r="590" hidden="true">
       <c r="A590" t="s" s="2">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="B590" t="s" s="2">
         <v>605</v>
@@ -64741,7 +64739,7 @@
     </row>
     <row r="591" hidden="true">
       <c r="A591" t="s" s="2">
-        <v>1128</v>
+        <v>1129</v>
       </c>
       <c r="B591" t="s" s="2">
         <v>607</v>
@@ -64845,7 +64843,7 @@
     </row>
     <row r="592" hidden="true">
       <c r="A592" t="s" s="2">
-        <v>1129</v>
+        <v>1130</v>
       </c>
       <c r="B592" t="s" s="2">
         <v>611</v>
@@ -64947,7 +64945,7 @@
     </row>
     <row r="593" hidden="true">
       <c r="A593" t="s" s="2">
-        <v>1130</v>
+        <v>1131</v>
       </c>
       <c r="B593" t="s" s="2">
         <v>613</v>
@@ -65051,7 +65049,7 @@
     </row>
     <row r="594" hidden="true">
       <c r="A594" t="s" s="2">
-        <v>1131</v>
+        <v>1132</v>
       </c>
       <c r="B594" t="s" s="2">
         <v>615</v>
@@ -65155,7 +65153,7 @@
     </row>
     <row r="595" hidden="true">
       <c r="A595" t="s" s="2">
-        <v>1132</v>
+        <v>1133</v>
       </c>
       <c r="B595" t="s" s="2">
         <v>617</v>
@@ -65259,7 +65257,7 @@
     </row>
     <row r="596" hidden="true">
       <c r="A596" t="s" s="2">
-        <v>1133</v>
+        <v>1134</v>
       </c>
       <c r="B596" t="s" s="2">
         <v>597</v>
@@ -65275,7 +65273,7 @@
         <v>74</v>
       </c>
       <c r="G596" t="s" s="2">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H596" t="s" s="2">
         <v>73</v>
@@ -65363,7 +65361,7 @@
     </row>
     <row r="597" hidden="true">
       <c r="A597" t="s" s="2">
-        <v>1134</v>
+        <v>1135</v>
       </c>
       <c r="B597" t="s" s="2">
         <v>603</v>
@@ -65463,7 +65461,7 @@
     </row>
     <row r="598" hidden="true">
       <c r="A598" t="s" s="2">
-        <v>1135</v>
+        <v>1136</v>
       </c>
       <c r="B598" t="s" s="2">
         <v>605</v>
@@ -65565,7 +65563,7 @@
     </row>
     <row r="599" hidden="true">
       <c r="A599" t="s" s="2">
-        <v>1136</v>
+        <v>1137</v>
       </c>
       <c r="B599" t="s" s="2">
         <v>607</v>
@@ -65669,7 +65667,7 @@
     </row>
     <row r="600" hidden="true">
       <c r="A600" t="s" s="2">
-        <v>1137</v>
+        <v>1138</v>
       </c>
       <c r="B600" t="s" s="2">
         <v>611</v>
@@ -65771,7 +65769,7 @@
     </row>
     <row r="601" hidden="true">
       <c r="A601" t="s" s="2">
-        <v>1138</v>
+        <v>1139</v>
       </c>
       <c r="B601" t="s" s="2">
         <v>613</v>
@@ -65875,7 +65873,7 @@
     </row>
     <row r="602" hidden="true">
       <c r="A602" t="s" s="2">
-        <v>1139</v>
+        <v>1140</v>
       </c>
       <c r="B602" t="s" s="2">
         <v>615</v>
@@ -65979,7 +65977,7 @@
     </row>
     <row r="603" hidden="true">
       <c r="A603" t="s" s="2">
-        <v>1140</v>
+        <v>1141</v>
       </c>
       <c r="B603" t="s" s="2">
         <v>617</v>
@@ -66083,7 +66081,7 @@
     </row>
     <row r="604" hidden="true">
       <c r="A604" t="s" s="2">
-        <v>1141</v>
+        <v>1142</v>
       </c>
       <c r="B604" t="s" s="2">
         <v>597</v>
@@ -66099,7 +66097,7 @@
         <v>74</v>
       </c>
       <c r="G604" t="s" s="2">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H604" t="s" s="2">
         <v>73</v>
@@ -66187,7 +66185,7 @@
     </row>
     <row r="605" hidden="true">
       <c r="A605" t="s" s="2">
-        <v>1142</v>
+        <v>1143</v>
       </c>
       <c r="B605" t="s" s="2">
         <v>603</v>
@@ -66287,7 +66285,7 @@
     </row>
     <row r="606" hidden="true">
       <c r="A606" t="s" s="2">
-        <v>1143</v>
+        <v>1144</v>
       </c>
       <c r="B606" t="s" s="2">
         <v>605</v>
@@ -66389,7 +66387,7 @@
     </row>
     <row r="607" hidden="true">
       <c r="A607" t="s" s="2">
-        <v>1144</v>
+        <v>1145</v>
       </c>
       <c r="B607" t="s" s="2">
         <v>607</v>
@@ -66493,7 +66491,7 @@
     </row>
     <row r="608" hidden="true">
       <c r="A608" t="s" s="2">
-        <v>1145</v>
+        <v>1146</v>
       </c>
       <c r="B608" t="s" s="2">
         <v>611</v>
@@ -66595,7 +66593,7 @@
     </row>
     <row r="609" hidden="true">
       <c r="A609" t="s" s="2">
-        <v>1146</v>
+        <v>1147</v>
       </c>
       <c r="B609" t="s" s="2">
         <v>613</v>
@@ -66699,7 +66697,7 @@
     </row>
     <row r="610" hidden="true">
       <c r="A610" t="s" s="2">
-        <v>1147</v>
+        <v>1148</v>
       </c>
       <c r="B610" t="s" s="2">
         <v>615</v>
@@ -66803,7 +66801,7 @@
     </row>
     <row r="611" hidden="true">
       <c r="A611" t="s" s="2">
-        <v>1148</v>
+        <v>1149</v>
       </c>
       <c r="B611" t="s" s="2">
         <v>617</v>
@@ -66907,7 +66905,7 @@
     </row>
     <row r="612" hidden="true">
       <c r="A612" t="s" s="2">
-        <v>1149</v>
+        <v>1150</v>
       </c>
       <c r="B612" t="s" s="2">
         <v>597</v>
@@ -66923,7 +66921,7 @@
         <v>74</v>
       </c>
       <c r="G612" t="s" s="2">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H612" t="s" s="2">
         <v>73</v>
@@ -67011,7 +67009,7 @@
     </row>
     <row r="613" hidden="true">
       <c r="A613" t="s" s="2">
-        <v>1150</v>
+        <v>1151</v>
       </c>
       <c r="B613" t="s" s="2">
         <v>603</v>
@@ -67111,7 +67109,7 @@
     </row>
     <row r="614" hidden="true">
       <c r="A614" t="s" s="2">
-        <v>1151</v>
+        <v>1152</v>
       </c>
       <c r="B614" t="s" s="2">
         <v>605</v>
@@ -67213,7 +67211,7 @@
     </row>
     <row r="615" hidden="true">
       <c r="A615" t="s" s="2">
-        <v>1152</v>
+        <v>1153</v>
       </c>
       <c r="B615" t="s" s="2">
         <v>607</v>
@@ -67317,7 +67315,7 @@
     </row>
     <row r="616" hidden="true">
       <c r="A616" t="s" s="2">
-        <v>1153</v>
+        <v>1154</v>
       </c>
       <c r="B616" t="s" s="2">
         <v>611</v>
@@ -67419,7 +67417,7 @@
     </row>
     <row r="617" hidden="true">
       <c r="A617" t="s" s="2">
-        <v>1154</v>
+        <v>1155</v>
       </c>
       <c r="B617" t="s" s="2">
         <v>613</v>
@@ -67523,7 +67521,7 @@
     </row>
     <row r="618" hidden="true">
       <c r="A618" t="s" s="2">
-        <v>1155</v>
+        <v>1156</v>
       </c>
       <c r="B618" t="s" s="2">
         <v>615</v>
@@ -67627,7 +67625,7 @@
     </row>
     <row r="619" hidden="true">
       <c r="A619" t="s" s="2">
-        <v>1156</v>
+        <v>1157</v>
       </c>
       <c r="B619" t="s" s="2">
         <v>617</v>
@@ -67731,7 +67729,7 @@
     </row>
     <row r="620" hidden="true">
       <c r="A620" t="s" s="2">
-        <v>1157</v>
+        <v>1158</v>
       </c>
       <c r="B620" t="s" s="2">
         <v>597</v>
@@ -67747,7 +67745,7 @@
         <v>74</v>
       </c>
       <c r="G620" t="s" s="2">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H620" t="s" s="2">
         <v>73</v>
@@ -67835,7 +67833,7 @@
     </row>
     <row r="621" hidden="true">
       <c r="A621" t="s" s="2">
-        <v>1158</v>
+        <v>1159</v>
       </c>
       <c r="B621" t="s" s="2">
         <v>603</v>
@@ -67935,7 +67933,7 @@
     </row>
     <row r="622" hidden="true">
       <c r="A622" t="s" s="2">
-        <v>1159</v>
+        <v>1160</v>
       </c>
       <c r="B622" t="s" s="2">
         <v>605</v>
@@ -68037,7 +68035,7 @@
     </row>
     <row r="623" hidden="true">
       <c r="A623" t="s" s="2">
-        <v>1160</v>
+        <v>1161</v>
       </c>
       <c r="B623" t="s" s="2">
         <v>607</v>
@@ -68141,7 +68139,7 @@
     </row>
     <row r="624" hidden="true">
       <c r="A624" t="s" s="2">
-        <v>1161</v>
+        <v>1162</v>
       </c>
       <c r="B624" t="s" s="2">
         <v>611</v>
@@ -68243,7 +68241,7 @@
     </row>
     <row r="625" hidden="true">
       <c r="A625" t="s" s="2">
-        <v>1162</v>
+        <v>1163</v>
       </c>
       <c r="B625" t="s" s="2">
         <v>613</v>
@@ -68347,7 +68345,7 @@
     </row>
     <row r="626" hidden="true">
       <c r="A626" t="s" s="2">
-        <v>1163</v>
+        <v>1164</v>
       </c>
       <c r="B626" t="s" s="2">
         <v>615</v>
@@ -68451,7 +68449,7 @@
     </row>
     <row r="627" hidden="true">
       <c r="A627" t="s" s="2">
-        <v>1164</v>
+        <v>1165</v>
       </c>
       <c r="B627" t="s" s="2">
         <v>617</v>
@@ -68555,7 +68553,7 @@
     </row>
     <row r="628" hidden="true">
       <c r="A628" t="s" s="2">
-        <v>1165</v>
+        <v>1166</v>
       </c>
       <c r="B628" t="s" s="2">
         <v>597</v>
@@ -68571,7 +68569,7 @@
         <v>74</v>
       </c>
       <c r="G628" t="s" s="2">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H628" t="s" s="2">
         <v>73</v>
@@ -68659,7 +68657,7 @@
     </row>
     <row r="629" hidden="true">
       <c r="A629" t="s" s="2">
-        <v>1166</v>
+        <v>1167</v>
       </c>
       <c r="B629" t="s" s="2">
         <v>603</v>
@@ -68759,7 +68757,7 @@
     </row>
     <row r="630" hidden="true">
       <c r="A630" t="s" s="2">
-        <v>1167</v>
+        <v>1168</v>
       </c>
       <c r="B630" t="s" s="2">
         <v>605</v>
@@ -68861,7 +68859,7 @@
     </row>
     <row r="631" hidden="true">
       <c r="A631" t="s" s="2">
-        <v>1168</v>
+        <v>1169</v>
       </c>
       <c r="B631" t="s" s="2">
         <v>607</v>
@@ -68965,7 +68963,7 @@
     </row>
     <row r="632" hidden="true">
       <c r="A632" t="s" s="2">
-        <v>1169</v>
+        <v>1170</v>
       </c>
       <c r="B632" t="s" s="2">
         <v>611</v>
@@ -69067,7 +69065,7 @@
     </row>
     <row r="633" hidden="true">
       <c r="A633" t="s" s="2">
-        <v>1170</v>
+        <v>1171</v>
       </c>
       <c r="B633" t="s" s="2">
         <v>613</v>
@@ -69171,7 +69169,7 @@
     </row>
     <row r="634" hidden="true">
       <c r="A634" t="s" s="2">
-        <v>1171</v>
+        <v>1172</v>
       </c>
       <c r="B634" t="s" s="2">
         <v>615</v>
@@ -69275,7 +69273,7 @@
     </row>
     <row r="635" hidden="true">
       <c r="A635" t="s" s="2">
-        <v>1172</v>
+        <v>1173</v>
       </c>
       <c r="B635" t="s" s="2">
         <v>617</v>
@@ -69379,7 +69377,7 @@
     </row>
     <row r="636" hidden="true">
       <c r="A636" t="s" s="2">
-        <v>1173</v>
+        <v>1174</v>
       </c>
       <c r="B636" t="s" s="2">
         <v>597</v>
@@ -69395,7 +69393,7 @@
         <v>74</v>
       </c>
       <c r="G636" t="s" s="2">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H636" t="s" s="2">
         <v>73</v>
@@ -69483,7 +69481,7 @@
     </row>
     <row r="637" hidden="true">
       <c r="A637" t="s" s="2">
-        <v>1174</v>
+        <v>1175</v>
       </c>
       <c r="B637" t="s" s="2">
         <v>603</v>
@@ -69583,7 +69581,7 @@
     </row>
     <row r="638" hidden="true">
       <c r="A638" t="s" s="2">
-        <v>1175</v>
+        <v>1176</v>
       </c>
       <c r="B638" t="s" s="2">
         <v>605</v>
@@ -69685,7 +69683,7 @@
     </row>
     <row r="639" hidden="true">
       <c r="A639" t="s" s="2">
-        <v>1176</v>
+        <v>1177</v>
       </c>
       <c r="B639" t="s" s="2">
         <v>607</v>
@@ -69789,7 +69787,7 @@
     </row>
     <row r="640" hidden="true">
       <c r="A640" t="s" s="2">
-        <v>1177</v>
+        <v>1178</v>
       </c>
       <c r="B640" t="s" s="2">
         <v>611</v>
@@ -69891,7 +69889,7 @@
     </row>
     <row r="641" hidden="true">
       <c r="A641" t="s" s="2">
-        <v>1178</v>
+        <v>1179</v>
       </c>
       <c r="B641" t="s" s="2">
         <v>613</v>
@@ -69995,7 +69993,7 @@
     </row>
     <row r="642" hidden="true">
       <c r="A642" t="s" s="2">
-        <v>1179</v>
+        <v>1180</v>
       </c>
       <c r="B642" t="s" s="2">
         <v>615</v>
@@ -70099,7 +70097,7 @@
     </row>
     <row r="643" hidden="true">
       <c r="A643" t="s" s="2">
-        <v>1180</v>
+        <v>1181</v>
       </c>
       <c r="B643" t="s" s="2">
         <v>617</v>
@@ -70203,7 +70201,7 @@
     </row>
     <row r="644" hidden="true">
       <c r="A644" t="s" s="2">
-        <v>1181</v>
+        <v>1182</v>
       </c>
       <c r="B644" t="s" s="2">
         <v>597</v>
@@ -70219,7 +70217,7 @@
         <v>74</v>
       </c>
       <c r="G644" t="s" s="2">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H644" t="s" s="2">
         <v>73</v>
@@ -70307,7 +70305,7 @@
     </row>
     <row r="645" hidden="true">
       <c r="A645" t="s" s="2">
-        <v>1182</v>
+        <v>1183</v>
       </c>
       <c r="B645" t="s" s="2">
         <v>603</v>
@@ -70407,7 +70405,7 @@
     </row>
     <row r="646" hidden="true">
       <c r="A646" t="s" s="2">
-        <v>1183</v>
+        <v>1184</v>
       </c>
       <c r="B646" t="s" s="2">
         <v>605</v>
@@ -70509,7 +70507,7 @@
     </row>
     <row r="647" hidden="true">
       <c r="A647" t="s" s="2">
-        <v>1184</v>
+        <v>1185</v>
       </c>
       <c r="B647" t="s" s="2">
         <v>607</v>
@@ -70613,7 +70611,7 @@
     </row>
     <row r="648" hidden="true">
       <c r="A648" t="s" s="2">
-        <v>1185</v>
+        <v>1186</v>
       </c>
       <c r="B648" t="s" s="2">
         <v>611</v>
@@ -70715,7 +70713,7 @@
     </row>
     <row r="649" hidden="true">
       <c r="A649" t="s" s="2">
-        <v>1186</v>
+        <v>1187</v>
       </c>
       <c r="B649" t="s" s="2">
         <v>613</v>
@@ -70819,7 +70817,7 @@
     </row>
     <row r="650" hidden="true">
       <c r="A650" t="s" s="2">
-        <v>1187</v>
+        <v>1188</v>
       </c>
       <c r="B650" t="s" s="2">
         <v>615</v>
@@ -70923,7 +70921,7 @@
     </row>
     <row r="651" hidden="true">
       <c r="A651" t="s" s="2">
-        <v>1188</v>
+        <v>1189</v>
       </c>
       <c r="B651" t="s" s="2">
         <v>617</v>
@@ -71027,13 +71025,13 @@
     </row>
     <row r="652" hidden="true">
       <c r="A652" t="s" s="2">
-        <v>1189</v>
+        <v>1190</v>
       </c>
       <c r="B652" t="s" s="2">
         <v>597</v>
       </c>
       <c r="C652" t="s" s="2">
-        <v>1190</v>
+        <v>1191</v>
       </c>
       <c r="D652" t="s" s="2">
         <v>73</v>
@@ -71058,7 +71056,7 @@
         <v>140</v>
       </c>
       <c r="L652" t="s" s="2">
-        <v>1191</v>
+        <v>1192</v>
       </c>
       <c r="M652" t="s" s="2">
         <v>243</v>
@@ -71096,7 +71094,7 @@
       </c>
       <c r="Y652" s="2"/>
       <c r="Z652" t="s" s="2">
-        <v>1192</v>
+        <v>1193</v>
       </c>
       <c r="AA652" t="s" s="2">
         <v>73</v>
@@ -71131,13 +71129,13 @@
     </row>
     <row r="653" hidden="true">
       <c r="A653" t="s" s="2">
-        <v>1193</v>
+        <v>1194</v>
       </c>
       <c r="B653" t="s" s="2">
         <v>597</v>
       </c>
       <c r="C653" t="s" s="2">
-        <v>1067</v>
+        <v>1068</v>
       </c>
       <c r="D653" t="s" s="2">
         <v>73</v>
@@ -71162,7 +71160,7 @@
         <v>140</v>
       </c>
       <c r="L653" t="s" s="2">
-        <v>1194</v>
+        <v>1195</v>
       </c>
       <c r="M653" t="s" s="2">
         <v>243</v>
@@ -71200,7 +71198,7 @@
       </c>
       <c r="Y653" s="2"/>
       <c r="Z653" t="s" s="2">
-        <v>1195</v>
+        <v>1196</v>
       </c>
       <c r="AA653" t="s" s="2">
         <v>73</v>
@@ -71235,7 +71233,7 @@
     </row>
     <row r="654" hidden="true">
       <c r="A654" t="s" s="2">
-        <v>1196</v>
+        <v>1197</v>
       </c>
       <c r="B654" t="s" s="2">
         <v>761</v>
@@ -71339,7 +71337,7 @@
     </row>
     <row r="655" hidden="true">
       <c r="A655" t="s" s="2">
-        <v>1197</v>
+        <v>1198</v>
       </c>
       <c r="B655" t="s" s="2">
         <v>762</v>
@@ -71443,7 +71441,7 @@
     </row>
     <row r="656" hidden="true">
       <c r="A656" t="s" s="2">
-        <v>1198</v>
+        <v>1199</v>
       </c>
       <c r="B656" t="s" s="2">
         <v>766</v>
@@ -71545,10 +71543,10 @@
     </row>
     <row r="657" hidden="true">
       <c r="A657" t="s" s="2">
-        <v>1199</v>
+        <v>1200</v>
       </c>
       <c r="B657" t="s" s="2">
-        <v>1199</v>
+        <v>1200</v>
       </c>
       <c r="C657" s="2"/>
       <c r="D657" t="s" s="2">
@@ -71571,19 +71569,19 @@
         <v>73</v>
       </c>
       <c r="K657" t="s" s="2">
-        <v>1200</v>
+        <v>1201</v>
       </c>
       <c r="L657" t="s" s="2">
-        <v>1201</v>
+        <v>1202</v>
       </c>
       <c r="M657" t="s" s="2">
-        <v>1202</v>
+        <v>1203</v>
       </c>
       <c r="N657" t="s" s="2">
         <v>592</v>
       </c>
       <c r="O657" t="s" s="2">
-        <v>1203</v>
+        <v>1204</v>
       </c>
       <c r="P657" t="s" s="2">
         <v>73</v>
@@ -71612,7 +71610,7 @@
       </c>
       <c r="Y657" s="2"/>
       <c r="Z657" t="s" s="2">
-        <v>1204</v>
+        <v>1205</v>
       </c>
       <c r="AA657" t="s" s="2">
         <v>73</v>
@@ -71630,7 +71628,7 @@
         <v>73</v>
       </c>
       <c r="AF657" t="s" s="2">
-        <v>1199</v>
+        <v>1200</v>
       </c>
       <c r="AG657" t="s" s="2">
         <v>74</v>

</xml_diff>